<commit_message>
#3 Client and JLCPCB BOM Updated.
</commit_message>
<xml_diff>
--- a/Design Files/Industrial IOT development board-v1.0/BOM/JLCPCB-BOM-v1.0.xlsx
+++ b/Design Files/Industrial IOT development board-v1.0/BOM/JLCPCB-BOM-v1.0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="620" uniqueCount="501">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="616" uniqueCount="500">
   <si>
     <t>Comment</t>
   </si>
@@ -87,13 +87,13 @@
     <t>AZ4024-01G</t>
   </si>
   <si>
-    <t>AZ3005-01G</t>
+    <t>PESD5V0S1BA,115-ES</t>
   </si>
   <si>
     <t>SMBJ26A-13-F</t>
   </si>
   <si>
-    <t>AZ3003-01G</t>
+    <t>PESD3V3L1BA-N-ES</t>
   </si>
   <si>
     <t>PMEG4030ER</t>
@@ -135,10 +135,10 @@
     <t>1210L075/24PR</t>
   </si>
   <si>
-    <t>1206L300SLTHYR</t>
-  </si>
-  <si>
-    <t>0805L110SLYR</t>
+    <t>BSMD1206-300-6V</t>
+  </si>
+  <si>
+    <t>SMD0805B110TF</t>
   </si>
   <si>
     <t>0805L050WR</t>
@@ -216,7 +216,7 @@
     <t>DMT6007LFG-7</t>
   </si>
   <si>
-    <t>SI7611DN-T1-GE3</t>
+    <t>AOD4185-JSM</t>
   </si>
   <si>
     <t>MMBT3904M</t>
@@ -324,9 +324,6 @@
     <t>12K</t>
   </si>
   <si>
-    <t>560R</t>
-  </si>
-  <si>
     <t>133R</t>
   </si>
   <si>
@@ -405,7 +402,7 @@
     <t>TPS2378DDAR</t>
   </si>
   <si>
-    <t>THVD1449DR</t>
+    <t>SP3485EIM/TR</t>
   </si>
   <si>
     <t>32.768kHz</t>
@@ -687,7 +684,7 @@
     <t>R8, R27</t>
   </si>
   <si>
-    <t>R9, R23, R31, R32, R33, R34, R39, R41, R42, R43, R46, R52, R53, R54, R55, R64, R65, R68, R69, R72, R73, R76, R77</t>
+    <t>R9, R23, R31, R32, R33, R34, R39, R41, R42, R43, R46, R52, R53, R54, R55, R64, R65, R68, R69, R72, R73, R76, R77, R117, R120</t>
   </si>
   <si>
     <t>R11, R100</t>
@@ -783,9 +780,6 @@
     <t>R114</t>
   </si>
   <si>
-    <t>R117, R120</t>
-  </si>
-  <si>
     <t>R122</t>
   </si>
   <si>
@@ -900,7 +894,7 @@
     <t>Cap-0603</t>
   </si>
   <si>
-    <t>35SVPF120M</t>
+    <t>OVZ121M1VTR-1013</t>
   </si>
   <si>
     <t>Cap-1206</t>
@@ -927,6 +921,9 @@
     <t>SOD-123</t>
   </si>
   <si>
+    <t>SOD-323 (Bi-directional)</t>
+  </si>
+  <si>
     <t>SOD-123FL</t>
   </si>
   <si>
@@ -987,7 +984,7 @@
     <t>PowerDI-3333-8</t>
   </si>
   <si>
-    <t>PowerPAK® 1212-8</t>
+    <t>TO-252-2L</t>
   </si>
   <si>
     <t>SOT-723</t>
@@ -1023,9 +1020,6 @@
     <t>SOT-23-6</t>
   </si>
   <si>
-    <t>TO-252-2L</t>
-  </si>
-  <si>
     <t>7-VQFN-HR (2x2)</t>
   </si>
   <si>
@@ -1056,6 +1050,9 @@
     <t>8-SO PowerPad</t>
   </si>
   <si>
+    <t>SOP-8</t>
+  </si>
+  <si>
     <t>MC-146_</t>
   </si>
   <si>
@@ -1086,7 +1083,7 @@
     <t>C307348</t>
   </si>
   <si>
-    <t>C501341</t>
+    <t>C250089</t>
   </si>
   <si>
     <t>C907991</t>
@@ -1173,13 +1170,13 @@
     <t>C5571859</t>
   </si>
   <si>
-    <t>C7079241</t>
+    <t>C41409246</t>
   </si>
   <si>
     <t>C135062</t>
   </si>
   <si>
-    <t>-</t>
+    <t>C41409249</t>
   </si>
   <si>
     <t>C5366303</t>
@@ -1221,10 +1218,10 @@
     <t>C207045</t>
   </si>
   <si>
-    <t>C207041</t>
-  </si>
-  <si>
-    <t>C207024</t>
+    <t>C883136</t>
+  </si>
+  <si>
+    <t>C269107</t>
   </si>
   <si>
     <t>C14709</t>
@@ -1299,7 +1296,7 @@
     <t>C2802568</t>
   </si>
   <si>
-    <t>C506599</t>
+    <t>C18189874</t>
   </si>
   <si>
     <t>C2923360</t>
@@ -1320,7 +1317,7 @@
     <t>C122538</t>
   </si>
   <si>
-    <t>C853910</t>
+    <t>C276265</t>
   </si>
   <si>
     <t>C100048</t>
@@ -1425,9 +1422,6 @@
     <t>C114659</t>
   </si>
   <si>
-    <t>C163460</t>
-  </si>
-  <si>
     <t>C114640</t>
   </si>
   <si>
@@ -1506,7 +1500,7 @@
     <t>C337500</t>
   </si>
   <si>
-    <t>C3235059</t>
+    <t>C519086</t>
   </si>
   <si>
     <t>C3013800</t>
@@ -1522,6 +1516,9 @@
   </si>
   <si>
     <t>C137948</t>
+  </si>
+  <si>
+    <t>C207022</t>
   </si>
 </sst>
 </file>
@@ -1967,7 +1964,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:D155"/>
+  <dimension ref="A1:D154"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.7109375" style="1" bestFit="1" customWidth="1"/>
@@ -1981,13 +1978,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="24" x14ac:dyDescent="0.25">
@@ -1995,13 +1992,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -2009,13 +2006,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -2023,13 +2020,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -2037,13 +2034,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -2051,13 +2048,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -2065,13 +2062,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -2079,13 +2076,13 @@
         <v>1</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -2093,13 +2090,13 @@
         <v>7</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -2107,13 +2104,13 @@
         <v>8</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -2121,13 +2118,13 @@
         <v>9</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -2135,13 +2132,13 @@
         <v>10</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -2149,13 +2146,13 @@
         <v>5</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -2163,13 +2160,13 @@
         <v>9</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -2177,13 +2174,13 @@
         <v>7</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -2191,13 +2188,13 @@
         <v>6</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -2205,13 +2202,13 @@
         <v>3</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -2219,13 +2216,13 @@
         <v>11</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -2233,13 +2230,13 @@
         <v>8</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -2247,13 +2244,13 @@
         <v>5</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
@@ -2261,13 +2258,13 @@
         <v>12</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
@@ -2275,13 +2272,13 @@
         <v>4</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -2289,13 +2286,13 @@
         <v>13</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
@@ -2303,13 +2300,13 @@
         <v>14</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
@@ -2317,13 +2314,13 @@
         <v>9</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
@@ -2331,13 +2328,13 @@
         <v>15</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
@@ -2345,13 +2342,13 @@
         <v>1</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
@@ -2359,13 +2356,13 @@
         <v>16</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
@@ -2373,13 +2370,13 @@
         <v>17</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
@@ -2387,13 +2384,13 @@
         <v>18</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
@@ -2401,13 +2398,13 @@
         <v>19</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
@@ -2415,13 +2412,13 @@
         <v>10</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
@@ -2429,13 +2426,13 @@
         <v>2</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
@@ -2443,13 +2440,13 @@
         <v>13</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
@@ -2457,13 +2454,13 @@
         <v>8</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
@@ -2471,13 +2468,13 @@
         <v>20</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
@@ -2485,27 +2482,27 @@
         <v>21</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>383</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" ht="24" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
         <v>22</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
@@ -2513,27 +2510,27 @@
         <v>23</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" ht="24" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
         <v>24</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
@@ -2541,13 +2538,13 @@
         <v>25</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
@@ -2555,13 +2552,13 @@
         <v>26</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
@@ -2569,13 +2566,13 @@
         <v>27</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="24" x14ac:dyDescent="0.25">
@@ -2583,13 +2580,13 @@
         <v>28</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
@@ -2597,13 +2594,13 @@
         <v>29</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
@@ -2611,13 +2608,13 @@
         <v>30</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
@@ -2625,13 +2622,13 @@
         <v>31</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="48" spans="1:4" ht="24" x14ac:dyDescent="0.25">
@@ -2639,13 +2636,13 @@
         <v>32</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
@@ -2653,13 +2650,13 @@
         <v>33</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C49" s="7" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
@@ -2667,13 +2664,13 @@
         <v>34</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
@@ -2681,13 +2678,13 @@
         <v>35</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
@@ -2695,13 +2692,13 @@
         <v>36</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
@@ -2709,13 +2706,13 @@
         <v>37</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C53" s="7" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
@@ -2723,13 +2720,13 @@
         <v>38</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="D54" s="4" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
@@ -2737,13 +2734,13 @@
         <v>39</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
@@ -2751,13 +2748,13 @@
         <v>40</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="D56" s="4" t="s">
-        <v>40</v>
+        <v>499</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
@@ -2765,13 +2762,13 @@
         <v>41</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C57" s="7" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
@@ -2779,13 +2776,13 @@
         <v>42</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D58" s="4" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
@@ -2793,13 +2790,13 @@
         <v>43</v>
       </c>
       <c r="B59" s="6" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C59" s="7" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
@@ -2807,13 +2804,13 @@
         <v>44</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C60" s="5" t="s">
         <v>44</v>
       </c>
       <c r="D60" s="4" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
@@ -2821,13 +2818,13 @@
         <v>45</v>
       </c>
       <c r="B61" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C61" s="7" t="s">
         <v>45</v>
       </c>
       <c r="D61" s="6" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
@@ -2835,13 +2832,13 @@
         <v>46</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C62" s="5" t="s">
         <v>46</v>
       </c>
       <c r="D62" s="4" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
@@ -2849,13 +2846,13 @@
         <v>47</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C63" s="7" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="D63" s="6" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
@@ -2863,13 +2860,13 @@
         <v>48</v>
       </c>
       <c r="B64" s="4" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C64" s="5" t="s">
         <v>48</v>
       </c>
       <c r="D64" s="4" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
@@ -2877,13 +2874,13 @@
         <v>49</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C65" s="7" t="s">
         <v>49</v>
       </c>
       <c r="D65" s="6" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
@@ -2891,13 +2888,13 @@
         <v>50</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C66" s="5" t="s">
         <v>50</v>
       </c>
       <c r="D66" s="4" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
@@ -2905,13 +2902,13 @@
         <v>51</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C67" s="7" t="s">
         <v>51</v>
       </c>
       <c r="D67" s="6" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
@@ -2919,13 +2916,13 @@
         <v>52</v>
       </c>
       <c r="B68" s="4" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C68" s="5" t="s">
         <v>52</v>
       </c>
       <c r="D68" s="4" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
@@ -2933,13 +2930,13 @@
         <v>53</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C69" s="7" t="s">
         <v>53</v>
       </c>
       <c r="D69" s="6" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
@@ -2947,13 +2944,13 @@
         <v>54</v>
       </c>
       <c r="B70" s="4" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C70" s="5" t="s">
         <v>54</v>
       </c>
       <c r="D70" s="4" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
@@ -2961,13 +2958,13 @@
         <v>55</v>
       </c>
       <c r="B71" s="6" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C71" s="7" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="D71" s="6" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
@@ -2975,13 +2972,13 @@
         <v>56</v>
       </c>
       <c r="B72" s="4" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C72" s="5" t="s">
         <v>56</v>
       </c>
       <c r="D72" s="4" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
@@ -2989,13 +2986,13 @@
         <v>57</v>
       </c>
       <c r="B73" s="6" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C73" s="7" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="D73" s="6" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
@@ -3003,13 +3000,13 @@
         <v>58</v>
       </c>
       <c r="B74" s="4" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C74" s="5" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="D74" s="4" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
@@ -3017,13 +3014,13 @@
         <v>59</v>
       </c>
       <c r="B75" s="6" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C75" s="7" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="D75" s="6" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
@@ -3031,13 +3028,13 @@
         <v>60</v>
       </c>
       <c r="B76" s="4" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C76" s="5" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="D76" s="4" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
@@ -3045,13 +3042,13 @@
         <v>61</v>
       </c>
       <c r="B77" s="6" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C77" s="7" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="D77" s="6" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
@@ -3059,13 +3056,13 @@
         <v>62</v>
       </c>
       <c r="B78" s="4" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C78" s="5" t="s">
         <v>62</v>
       </c>
       <c r="D78" s="4" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
@@ -3073,13 +3070,13 @@
         <v>63</v>
       </c>
       <c r="B79" s="6" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C79" s="7" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="D79" s="6" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
@@ -3087,13 +3084,13 @@
         <v>64</v>
       </c>
       <c r="B80" s="4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C80" s="5" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="D80" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
@@ -3101,13 +3098,13 @@
         <v>65</v>
       </c>
       <c r="B81" s="6" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C81" s="7" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="D81" s="6" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
@@ -3115,13 +3112,13 @@
         <v>66</v>
       </c>
       <c r="B82" s="4" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C82" s="5" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="D82" s="4" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
@@ -3129,13 +3126,13 @@
         <v>67</v>
       </c>
       <c r="B83" s="6" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C83" s="7" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="D83" s="6" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
@@ -3143,13 +3140,13 @@
         <v>68</v>
       </c>
       <c r="B84" s="4" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C84" s="5" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="D84" s="4" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
@@ -3157,13 +3154,13 @@
         <v>69</v>
       </c>
       <c r="B85" s="6" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C85" s="7" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="D85" s="6" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
@@ -3171,13 +3168,13 @@
         <v>70</v>
       </c>
       <c r="B86" s="4" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C86" s="5" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D86" s="4" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
@@ -3185,13 +3182,13 @@
         <v>70</v>
       </c>
       <c r="B87" s="6" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C87" s="7" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D87" s="6" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
@@ -3199,13 +3196,13 @@
         <v>71</v>
       </c>
       <c r="B88" s="4" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C88" s="5" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D88" s="4" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
@@ -3213,13 +3210,13 @@
         <v>70</v>
       </c>
       <c r="B89" s="6" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C89" s="7" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D89" s="6" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
@@ -3227,13 +3224,13 @@
         <v>72</v>
       </c>
       <c r="B90" s="4" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C90" s="5" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D90" s="4" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
@@ -3241,13 +3238,13 @@
         <v>73</v>
       </c>
       <c r="B91" s="6" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C91" s="7" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D91" s="6" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="92" spans="1:4" ht="36" x14ac:dyDescent="0.25">
@@ -3255,13 +3252,13 @@
         <v>74</v>
       </c>
       <c r="B92" s="4" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C92" s="5" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D92" s="4" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
@@ -3269,13 +3266,13 @@
         <v>75</v>
       </c>
       <c r="B93" s="6" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C93" s="7" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D93" s="6" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
@@ -3283,13 +3280,13 @@
         <v>76</v>
       </c>
       <c r="B94" s="4" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C94" s="5" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D94" s="4" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
@@ -3297,13 +3294,13 @@
         <v>77</v>
       </c>
       <c r="B95" s="6" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C95" s="7" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D95" s="6" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
@@ -3311,13 +3308,13 @@
         <v>78</v>
       </c>
       <c r="B96" s="4" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C96" s="5" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D96" s="4" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
@@ -3325,13 +3322,13 @@
         <v>79</v>
       </c>
       <c r="B97" s="6" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C97" s="7" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D97" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
@@ -3339,13 +3336,13 @@
         <v>80</v>
       </c>
       <c r="B98" s="4" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C98" s="5" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D98" s="4" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
     </row>
     <row r="99" spans="1:4" ht="24" x14ac:dyDescent="0.25">
@@ -3353,13 +3350,13 @@
         <v>81</v>
       </c>
       <c r="B99" s="6" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C99" s="7" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D99" s="6" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
@@ -3367,13 +3364,13 @@
         <v>82</v>
       </c>
       <c r="B100" s="4" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C100" s="5" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D100" s="4" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
@@ -3381,13 +3378,13 @@
         <v>83</v>
       </c>
       <c r="B101" s="4" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C101" s="5" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D101" s="4" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
@@ -3395,13 +3392,13 @@
         <v>84</v>
       </c>
       <c r="B102" s="6" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C102" s="7" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D102" s="6" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
@@ -3409,13 +3406,13 @@
         <v>84</v>
       </c>
       <c r="B103" s="4" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C103" s="5" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D103" s="4" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
@@ -3423,13 +3420,13 @@
         <v>85</v>
       </c>
       <c r="B104" s="6" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C104" s="7" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D104" s="6" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
@@ -3437,13 +3434,13 @@
         <v>82</v>
       </c>
       <c r="B105" s="4" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C105" s="5" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="D105" s="4" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
@@ -3451,13 +3448,13 @@
         <v>86</v>
       </c>
       <c r="B106" s="6" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C106" s="7" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D106" s="6" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
@@ -3465,13 +3462,13 @@
         <v>87</v>
       </c>
       <c r="B107" s="4" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C107" s="5" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D107" s="4" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
@@ -3479,13 +3476,13 @@
         <v>88</v>
       </c>
       <c r="B108" s="6" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C108" s="7" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D108" s="6" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
@@ -3493,13 +3490,13 @@
         <v>89</v>
       </c>
       <c r="B109" s="4" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C109" s="5" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D109" s="4" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
@@ -3507,13 +3504,13 @@
         <v>90</v>
       </c>
       <c r="B110" s="6" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C110" s="7" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D110" s="6" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
@@ -3521,13 +3518,13 @@
         <v>91</v>
       </c>
       <c r="B111" s="4" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C111" s="5" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D111" s="4" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
@@ -3535,13 +3532,13 @@
         <v>92</v>
       </c>
       <c r="B112" s="6" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C112" s="7" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D112" s="6" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
@@ -3549,13 +3546,13 @@
         <v>85</v>
       </c>
       <c r="B113" s="4" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C113" s="5" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D113" s="4" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
@@ -3563,13 +3560,13 @@
         <v>93</v>
       </c>
       <c r="B114" s="6" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C114" s="7" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D114" s="6" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
@@ -3577,13 +3574,13 @@
         <v>75</v>
       </c>
       <c r="B115" s="4" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C115" s="5" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D115" s="4" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
@@ -3591,13 +3588,13 @@
         <v>94</v>
       </c>
       <c r="B116" s="6" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C116" s="7" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D116" s="6" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
@@ -3605,13 +3602,13 @@
         <v>81</v>
       </c>
       <c r="B117" s="4" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C117" s="5" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="D117" s="4" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
@@ -3619,13 +3616,13 @@
         <v>95</v>
       </c>
       <c r="B118" s="6" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C118" s="7" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D118" s="6" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
@@ -3633,13 +3630,13 @@
         <v>96</v>
       </c>
       <c r="B119" s="4" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C119" s="5" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="D119" s="4" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
@@ -3647,13 +3644,13 @@
         <v>97</v>
       </c>
       <c r="B120" s="6" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C120" s="7" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D120" s="6" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
@@ -3661,13 +3658,13 @@
         <v>98</v>
       </c>
       <c r="B121" s="4" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C121" s="5" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D121" s="4" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
@@ -3675,13 +3672,13 @@
         <v>99</v>
       </c>
       <c r="B122" s="6" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C122" s="7" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D122" s="6" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
@@ -3689,41 +3686,41 @@
         <v>100</v>
       </c>
       <c r="B123" s="4" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="C123" s="5" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D123" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" s="6" t="s">
-        <v>101</v>
+        <v>41</v>
       </c>
       <c r="B124" s="6" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C124" s="7" t="s">
         <v>327</v>
       </c>
       <c r="D124" s="6" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" s="4" t="s">
-        <v>41</v>
+        <v>101</v>
       </c>
       <c r="B125" s="4" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C125" s="5" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="D125" s="4" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.25">
@@ -3731,13 +3728,13 @@
         <v>102</v>
       </c>
       <c r="B126" s="6" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="C126" s="7" t="s">
         <v>327</v>
       </c>
       <c r="D126" s="6" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.25">
@@ -3745,41 +3742,41 @@
         <v>103</v>
       </c>
       <c r="B127" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="C127" s="5" t="s">
+        <v>327</v>
+      </c>
+      <c r="D127" s="4" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A128" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="B128" s="4" t="s">
         <v>257</v>
       </c>
-      <c r="C127" s="5" t="s">
-        <v>328</v>
-      </c>
-      <c r="D127" s="4" t="s">
-        <v>471</v>
-      </c>
-    </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A128" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="B128" s="6" t="s">
-        <v>258</v>
-      </c>
-      <c r="C128" s="7" t="s">
-        <v>328</v>
-      </c>
-      <c r="D128" s="6" t="s">
-        <v>499</v>
+      <c r="C128" s="5" t="s">
+        <v>330</v>
+      </c>
+      <c r="D128" s="4" t="s">
+        <v>470</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" s="6" t="s">
-        <v>84</v>
+        <v>104</v>
       </c>
       <c r="B129" s="6" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="C129" s="7" t="s">
-        <v>331</v>
+        <v>104</v>
       </c>
       <c r="D129" s="6" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.25">
@@ -3787,13 +3784,13 @@
         <v>105</v>
       </c>
       <c r="B130" s="4" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C130" s="5" t="s">
         <v>105</v>
       </c>
       <c r="D130" s="4" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.25">
@@ -3801,13 +3798,13 @@
         <v>106</v>
       </c>
       <c r="B131" s="6" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C131" s="7" t="s">
         <v>106</v>
       </c>
       <c r="D131" s="6" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.25">
@@ -3815,13 +3812,13 @@
         <v>107</v>
       </c>
       <c r="B132" s="4" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C132" s="5" t="s">
         <v>107</v>
       </c>
       <c r="D132" s="4" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.25">
@@ -3829,13 +3826,13 @@
         <v>108</v>
       </c>
       <c r="B133" s="6" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C133" s="7" t="s">
         <v>108</v>
       </c>
       <c r="D133" s="6" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.25">
@@ -3843,13 +3840,13 @@
         <v>109</v>
       </c>
       <c r="B134" s="4" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C134" s="5" t="s">
         <v>109</v>
       </c>
       <c r="D134" s="4" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.25">
@@ -3857,13 +3854,13 @@
         <v>110</v>
       </c>
       <c r="B135" s="6" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="C135" s="7" t="s">
-        <v>110</v>
+        <v>331</v>
       </c>
       <c r="D135" s="6" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.25">
@@ -3871,13 +3868,13 @@
         <v>111</v>
       </c>
       <c r="B136" s="4" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C136" s="5" t="s">
         <v>332</v>
       </c>
       <c r="D136" s="4" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.25">
@@ -3885,13 +3882,13 @@
         <v>112</v>
       </c>
       <c r="B137" s="6" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="C137" s="7" t="s">
-        <v>333</v>
+        <v>321</v>
       </c>
       <c r="D137" s="6" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.25">
@@ -3899,13 +3896,13 @@
         <v>113</v>
       </c>
       <c r="B138" s="4" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C138" s="5" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="D138" s="4" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.25">
@@ -3913,13 +3910,13 @@
         <v>114</v>
       </c>
       <c r="B139" s="6" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C139" s="7" t="s">
         <v>333</v>
       </c>
       <c r="D139" s="6" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.25">
@@ -3927,69 +3924,69 @@
         <v>115</v>
       </c>
       <c r="B140" s="4" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C140" s="5" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D140" s="4" t="s">
-        <v>483</v>
-      </c>
-    </row>
-    <row r="141" spans="1:4" x14ac:dyDescent="0.25">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="141" spans="1:4" ht="24" x14ac:dyDescent="0.25">
       <c r="A141" s="6" t="s">
         <v>116</v>
       </c>
       <c r="B141" s="6" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C141" s="7" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="D141" s="6" t="s">
-        <v>498</v>
-      </c>
-    </row>
-    <row r="142" spans="1:4" ht="24" x14ac:dyDescent="0.25">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142" s="4" t="s">
         <v>117</v>
       </c>
       <c r="B142" s="4" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C142" s="5" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D142" s="4" t="s">
-        <v>484</v>
-      </c>
-    </row>
-    <row r="143" spans="1:4" x14ac:dyDescent="0.25">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="143" spans="1:4" ht="24" x14ac:dyDescent="0.25">
       <c r="A143" s="6" t="s">
         <v>118</v>
       </c>
       <c r="B143" s="6" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="C143" s="7" t="s">
-        <v>338</v>
+        <v>305</v>
       </c>
       <c r="D143" s="6" t="s">
-        <v>485</v>
-      </c>
-    </row>
-    <row r="144" spans="1:4" ht="24" x14ac:dyDescent="0.25">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="144" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A144" s="4" t="s">
         <v>119</v>
       </c>
       <c r="B144" s="4" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C144" s="5" t="s">
-        <v>306</v>
+        <v>337</v>
       </c>
       <c r="D144" s="4" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.25">
@@ -3997,13 +3994,13 @@
         <v>120</v>
       </c>
       <c r="B145" s="6" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C145" s="7" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D145" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.25">
@@ -4011,13 +4008,13 @@
         <v>121</v>
       </c>
       <c r="B146" s="4" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C146" s="5" t="s">
-        <v>340</v>
+        <v>121</v>
       </c>
       <c r="D146" s="4" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.25">
@@ -4025,13 +4022,13 @@
         <v>122</v>
       </c>
       <c r="B147" s="6" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C147" s="7" t="s">
-        <v>122</v>
+        <v>339</v>
       </c>
       <c r="D147" s="6" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.25">
@@ -4039,13 +4036,13 @@
         <v>123</v>
       </c>
       <c r="B148" s="4" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C148" s="5" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="D148" s="4" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.25">
@@ -4053,13 +4050,13 @@
         <v>124</v>
       </c>
       <c r="B149" s="6" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C149" s="7" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D149" s="6" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.25">
@@ -4067,13 +4064,13 @@
         <v>125</v>
       </c>
       <c r="B150" s="4" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C150" s="5" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="D150" s="4" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.25">
@@ -4081,13 +4078,13 @@
         <v>126</v>
       </c>
       <c r="B151" s="6" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C151" s="7" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="D151" s="6" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.25">
@@ -4095,27 +4092,27 @@
         <v>127</v>
       </c>
       <c r="B152" s="4" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C152" s="5" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="D152" s="4" t="s">
-        <v>494</v>
-      </c>
-    </row>
-    <row r="153" spans="1:4" ht="24" x14ac:dyDescent="0.25">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="153" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A153" s="6" t="s">
         <v>128</v>
       </c>
       <c r="B153" s="6" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C153" s="7" t="s">
-        <v>306</v>
+        <v>344</v>
       </c>
       <c r="D153" s="6" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.25">
@@ -4123,27 +4120,13 @@
         <v>129</v>
       </c>
       <c r="B154" s="4" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C154" s="5" t="s">
         <v>345</v>
       </c>
       <c r="D154" s="4" t="s">
-        <v>496</v>
-      </c>
-    </row>
-    <row r="155" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A155" s="6" t="s">
-        <v>130</v>
-      </c>
-      <c r="B155" s="6" t="s">
-        <v>285</v>
-      </c>
-      <c r="C155" s="7" t="s">
-        <v>346</v>
-      </c>
-      <c r="D155" s="6" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
     </row>
   </sheetData>

</xml_diff>